<commit_message>
Refactor analysis notebook and update README
</commit_message>
<xml_diff>
--- a/depth_analysis_topPercent.xlsx
+++ b/depth_analysis_topPercent.xlsx
@@ -455,7 +455,7 @@
         <v>-884.95</v>
       </c>
       <c r="B2" t="n">
-        <v>1.903304739996208</v>
+        <v>1.581293955660086</v>
       </c>
       <c r="C2" t="n">
         <v>23</v>
@@ -469,7 +469,7 @@
         <v>-874.95</v>
       </c>
       <c r="B3" t="n">
-        <v>1.986878587439439</v>
+        <v>1.983046647949812</v>
       </c>
       <c r="C3" t="n">
         <v>33</v>
@@ -483,7 +483,7 @@
         <v>-864.95</v>
       </c>
       <c r="B4" t="n">
-        <v>1.995664999118309</v>
+        <v>1.978858102040349</v>
       </c>
       <c r="C4" t="n">
         <v>33</v>
@@ -497,13 +497,13 @@
         <v>-854.95</v>
       </c>
       <c r="B5" t="n">
-        <v>1.928659348959487</v>
+        <v>2.056893435591113</v>
       </c>
       <c r="C5" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D5" t="n">
-        <v>3.41</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="6">
@@ -511,13 +511,13 @@
         <v>-844.95</v>
       </c>
       <c r="B6" t="n">
-        <v>2.013404493926854</v>
+        <v>2.003502551055158</v>
       </c>
       <c r="C6" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="D6" t="n">
-        <v>5.81</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="7">
@@ -525,7 +525,7 @@
         <v>-834.95</v>
       </c>
       <c r="B7" t="n">
-        <v>2.011562244105741</v>
+        <v>1.989559133058108</v>
       </c>
       <c r="C7" t="n">
         <v>44</v>
@@ -539,13 +539,13 @@
         <v>-824.95</v>
       </c>
       <c r="B8" t="n">
-        <v>1.983149791387759</v>
+        <v>2.02321787807761</v>
       </c>
       <c r="C8" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D8" t="n">
-        <v>3.41</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="9">
@@ -553,13 +553,13 @@
         <v>-814.95</v>
       </c>
       <c r="B9" t="n">
-        <v>2.022750939220819</v>
+        <v>1.995152763960439</v>
       </c>
       <c r="C9" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D9" t="n">
-        <v>3.41</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="10">
@@ -567,13 +567,13 @@
         <v>-804.95</v>
       </c>
       <c r="B10" t="n">
-        <v>2.006077166841798</v>
+        <v>1.998727673418004</v>
       </c>
       <c r="C10" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D10" t="n">
-        <v>3.41</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="11">
@@ -581,7 +581,7 @@
         <v>-794.95</v>
       </c>
       <c r="B11" t="n">
-        <v>1.988661440292017</v>
+        <v>1.915251517316802</v>
       </c>
       <c r="C11" t="n">
         <v>33</v>
@@ -595,13 +595,13 @@
         <v>-784.95</v>
       </c>
       <c r="B12" t="n">
-        <v>2.000580762054733</v>
+        <v>2.014955198246541</v>
       </c>
       <c r="C12" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D12" t="n">
-        <v>3.41</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="13">
@@ -609,13 +609,13 @@
         <v>-774.95</v>
       </c>
       <c r="B13" t="n">
-        <v>1.981174332058023</v>
+        <v>2.019934779684203</v>
       </c>
       <c r="C13" t="n">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="D13" t="n">
-        <v>4.45</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="14">
@@ -623,13 +623,13 @@
         <v>-764.95</v>
       </c>
       <c r="B14" t="n">
-        <v>2.009618822382897</v>
+        <v>1.852359275135956</v>
       </c>
       <c r="C14" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D14" t="n">
-        <v>2.59</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="15">
@@ -637,13 +637,13 @@
         <v>-754.95</v>
       </c>
       <c r="B15" t="n">
-        <v>2.009339804317092</v>
+        <v>2.027016228854273</v>
       </c>
       <c r="C15" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D15" t="n">
-        <v>2.59</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="16">
@@ -651,13 +651,13 @@
         <v>-744.95</v>
       </c>
       <c r="B16" t="n">
-        <v>1.653492077572112</v>
+        <v>1.439867715897145</v>
       </c>
       <c r="C16" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="D16" t="n">
-        <v>4.45</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="17">
@@ -665,7 +665,7 @@
         <v>-734.95</v>
       </c>
       <c r="B17" t="n">
-        <v>1.666907799355008</v>
+        <v>1.416366795513494</v>
       </c>
       <c r="C17" t="n">
         <v>49</v>
@@ -679,7 +679,7 @@
         <v>-724.95</v>
       </c>
       <c r="B18" t="n">
-        <v>1.562860782214803</v>
+        <v>1.313883943546284</v>
       </c>
       <c r="C18" t="n">
         <v>49</v>
@@ -693,13 +693,13 @@
         <v>-714.95</v>
       </c>
       <c r="B19" t="n">
-        <v>1.520323928487815</v>
+        <v>1.277215669869523</v>
       </c>
       <c r="C19" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="D19" t="n">
-        <v>1.68</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="20">
@@ -707,7 +707,7 @@
         <v>-704.95</v>
       </c>
       <c r="B20" t="n">
-        <v>1.426536201430606</v>
+        <v>1.1092880675901</v>
       </c>
       <c r="C20" t="n">
         <v>49</v>
@@ -721,7 +721,7 @@
         <v>-694.95</v>
       </c>
       <c r="B21" t="n">
-        <v>1.400742107238836</v>
+        <v>1.150598082263472</v>
       </c>
       <c r="C21" t="n">
         <v>49</v>
@@ -735,7 +735,7 @@
         <v>-684.95</v>
       </c>
       <c r="B22" t="n">
-        <v>1.240245058394525</v>
+        <v>1.095854999002241</v>
       </c>
       <c r="C22" t="n">
         <v>49</v>

</xml_diff>